<commit_message>
fixed turbine rotor sign error
</commit_message>
<xml_diff>
--- a/xjep_turbojet/turbine.xlsx
+++ b/xjep_turbojet/turbine.xlsx
@@ -491,7 +491,7 @@
         <v>536.416862571631</v>
       </c>
       <c r="D4" t="n">
-        <v>451.2991562877635</v>
+        <v>-451.2991562877635</v>
       </c>
     </row>
     <row r="5">
@@ -507,7 +507,7 @@
         <v>371.6263670071519</v>
       </c>
       <c r="D5" t="n">
-        <v>391.6198720615981</v>
+        <v>904.1398278688348</v>
       </c>
     </row>
     <row r="6">
@@ -523,7 +523,7 @@
         <v>190.8767288616049</v>
       </c>
       <c r="D6" t="n">
-        <v>83.41529538725172</v>
+        <v>-819.1830171882754</v>
       </c>
     </row>
     <row r="7">
@@ -571,7 +571,7 @@
         <v>0.6190475126105447</v>
       </c>
       <c r="D9" t="n">
-        <v>1.009863609763522</v>
+        <v>2.331490242045164</v>
       </c>
     </row>
     <row r="10">
@@ -587,7 +587,7 @@
         <v>59.27159396098239</v>
       </c>
       <c r="D10" t="n">
-        <v>49.70712822060125</v>
+        <v>-49.70712822060125</v>
       </c>
     </row>
     <row r="11">
@@ -603,7 +603,7 @@
         <v>30.90561674233874</v>
       </c>
       <c r="D11" t="n">
-        <v>12.29825742570211</v>
+        <v>-64.96314595993412</v>
       </c>
     </row>
     <row r="12">
@@ -717,7 +717,7 @@
         <v>534.0686604268027</v>
       </c>
       <c r="D20" t="n">
-        <v>433.9031814722879</v>
+        <v>-433.9031814722879</v>
       </c>
     </row>
     <row r="21">
@@ -733,7 +733,7 @@
         <v>369.6548263151458</v>
       </c>
       <c r="D21" t="n">
-        <v>386.052644333906</v>
+        <v>901.7423957773889</v>
       </c>
     </row>
     <row r="22">
@@ -749,7 +749,7 @@
         <v>187.0092499959637</v>
       </c>
       <c r="D22" t="n">
-        <v>51.27018147228796</v>
+        <v>-816.5361814722879</v>
       </c>
     </row>
     <row r="23">
@@ -797,7 +797,7 @@
         <v>0.6157633609201633</v>
       </c>
       <c r="D25" t="n">
-        <v>0.9955074927976847</v>
+        <v>2.325308024035425</v>
       </c>
     </row>
     <row r="26">
@@ -813,7 +813,7 @@
         <v>59.16107092132572</v>
       </c>
       <c r="D26" t="n">
-        <v>48.59287643690928</v>
+        <v>-48.59287643690928</v>
       </c>
     </row>
     <row r="27">
@@ -829,7 +829,7 @@
         <v>30.3912715428547</v>
       </c>
       <c r="D27" t="n">
-        <v>7.631781651699313</v>
+        <v>-64.89197315792033</v>
       </c>
     </row>
     <row r="28">
@@ -943,7 +943,7 @@
         <v>531.7409275130885</v>
       </c>
       <c r="D36" t="n">
-        <v>417.7985362213774</v>
+        <v>-417.7985362213774</v>
       </c>
     </row>
     <row r="37">
@@ -959,7 +959,7 @@
         <v>367.7235882130061</v>
       </c>
       <c r="D37" t="n">
-        <v>383.1772983364733</v>
+        <v>900.5151559555134</v>
       </c>
     </row>
     <row r="38">
@@ -975,7 +975,7 @@
         <v>183.1622403614367</v>
       </c>
       <c r="D38" t="n">
-        <v>20.4163971218893</v>
+        <v>-815.1806753208656</v>
       </c>
     </row>
     <row r="39">
@@ -1023,7 +1023,7 @@
         <v>0.6125463444500556</v>
       </c>
       <c r="D41" t="n">
-        <v>0.9880928861971551</v>
+        <v>2.322143361246378</v>
       </c>
     </row>
     <row r="42">
@@ -1039,7 +1039,7 @@
         <v>59.05080187210248</v>
       </c>
       <c r="D42" t="n">
-        <v>47.51557056437037</v>
+        <v>-47.51557056437037</v>
       </c>
     </row>
     <row r="43">
@@ -1055,7 +1055,7 @@
         <v>29.87421848879016</v>
       </c>
       <c r="D43" t="n">
-        <v>3.0542717184137</v>
+        <v>-64.85537720482064</v>
       </c>
     </row>
     <row r="44">
@@ -1230,7 +1230,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1308,6 +1308,38 @@
         <v>0.02496742353022317</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>stator NOB</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>159</v>
+      </c>
+      <c r="C6" t="n">
+        <v>159</v>
+      </c>
+      <c r="D6" t="n">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>rotor NOB</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>79</v>
+      </c>
+      <c r="C7" t="n">
+        <v>79</v>
+      </c>
+      <c r="D7" t="n">
+        <v>79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fixed various bugs and added more parameters to the excel output
</commit_message>
<xml_diff>
--- a/xjep_turbojet/turbine.xlsx
+++ b/xjep_turbojet/turbine.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D49"/>
+  <dimension ref="A1:D52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,10 +456,10 @@
         <v>318.8608333333333</v>
       </c>
       <c r="C2" t="n">
-        <v>624.0314747552561</v>
+        <v>641.6967391141203</v>
       </c>
       <c r="D2" t="n">
-        <v>591.6746920014808</v>
+        <v>468.048116610378</v>
       </c>
     </row>
     <row r="3">
@@ -488,10 +488,10 @@
         <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>536.416862571631</v>
+        <v>556.8684530081297</v>
       </c>
       <c r="D4" t="n">
-        <v>-451.2991562877635</v>
+        <v>-269.5570937176798</v>
       </c>
     </row>
     <row r="5">
@@ -504,10 +504,10 @@
         <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>371.6263670071519</v>
+        <v>389.6878070433993</v>
       </c>
       <c r="D5" t="n">
-        <v>904.1398278688348</v>
+        <v>677.9017718664238</v>
       </c>
     </row>
     <row r="6">
@@ -520,10 +520,10 @@
         <v>0</v>
       </c>
       <c r="C6" t="n">
-        <v>190.8767288616049</v>
+        <v>224.0186508402053</v>
       </c>
       <c r="D6" t="n">
-        <v>-819.1830171882754</v>
+        <v>-559.5916364730954</v>
       </c>
     </row>
     <row r="7">
@@ -536,10 +536,10 @@
         <v>0</v>
       </c>
       <c r="C7" t="n">
-        <v>345.5401337100261</v>
+        <v>332.8498021679244</v>
       </c>
       <c r="D7" t="n">
-        <v>367.8838609005118</v>
+        <v>290.0345427554155</v>
       </c>
     </row>
     <row r="8">
@@ -549,13 +549,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.6742997789701619</v>
+        <v>0.5023026870006502</v>
       </c>
       <c r="C8" t="n">
-        <v>1.039498718427847</v>
+        <v>1.068925150273982</v>
       </c>
       <c r="D8" t="n">
-        <v>1.525741625737401</v>
+        <v>1.120609616342567</v>
       </c>
     </row>
     <row r="9">
@@ -568,10 +568,10 @@
         <v>0</v>
       </c>
       <c r="C9" t="n">
-        <v>0.6190475126105447</v>
+        <v>0.6491338857025494</v>
       </c>
       <c r="D9" t="n">
-        <v>2.331490242045164</v>
+        <v>1.623045190290881</v>
       </c>
     </row>
     <row r="10">
@@ -584,10 +584,10 @@
         <v>0</v>
       </c>
       <c r="C10" t="n">
-        <v>59.27159396098239</v>
+        <v>60.20470594438805</v>
       </c>
       <c r="D10" t="n">
-        <v>-49.70712822060125</v>
+        <v>-35.16390951060599</v>
       </c>
     </row>
     <row r="11">
@@ -600,10 +600,10 @@
         <v>0</v>
       </c>
       <c r="C11" t="n">
-        <v>30.90561674233874</v>
+        <v>35.09031690804215</v>
       </c>
       <c r="D11" t="n">
-        <v>-64.96314595993412</v>
+        <v>-55.63677914937897</v>
       </c>
     </row>
     <row r="12">
@@ -616,10 +616,10 @@
         <v>1012.274989914663</v>
       </c>
       <c r="C12" t="n">
-        <v>764.0040338620881</v>
+        <v>744.7118374335867</v>
       </c>
       <c r="D12" t="n">
-        <v>477.8957999745127</v>
+        <v>676.1336498097077</v>
       </c>
     </row>
     <row r="13">
@@ -629,20 +629,30 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>269971.8007849224</v>
+        <v>269.9718031524023</v>
       </c>
       <c r="C13" t="n">
-        <v>83484.76451029717</v>
+        <v>77.70112712892625</v>
       </c>
       <c r="D13" t="n">
-        <v>14061.97890106564</v>
+        <v>54.06219056033665</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr"/>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>reaction</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0.6276409011903206</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.6276409011903206</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.6276409011903206</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr"/>
@@ -657,224 +667,234 @@
       <c r="D16" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="inlineStr">
+      <c r="A17" t="inlineStr"/>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="inlineStr">
         <is>
           <t>radius 1</t>
         </is>
       </c>
-      <c r="B17" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="C17" s="1" t="n">
+      <c r="B18" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D17" s="1" t="n">
+      <c r="D18" s="1" t="n">
         <v>2</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>318.8608333333333</v>
-      </c>
-      <c r="C18" t="n">
-        <v>622.0141196822683</v>
-      </c>
-      <c r="D18" t="n">
-        <v>578.5153270059258</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Vax</t>
+          <t>V</t>
         </is>
       </c>
       <c r="B19" t="n">
         <v>318.8608333333333</v>
       </c>
       <c r="C19" t="n">
-        <v>318.8608333333333</v>
+        <v>622.0141196822682</v>
       </c>
       <c r="D19" t="n">
-        <v>382.633</v>
+        <v>433.7695896501622</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Vu</t>
+          <t>Vax</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0</v>
+        <v>318.8608333333333</v>
       </c>
       <c r="C20" t="n">
-        <v>534.0686604268027</v>
+        <v>318.8608333333333</v>
       </c>
       <c r="D20" t="n">
-        <v>-433.9031814722879</v>
+        <v>382.633</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>Vu</t>
         </is>
       </c>
       <c r="B21" t="n">
         <v>0</v>
       </c>
       <c r="C21" t="n">
-        <v>369.6548263151458</v>
+        <v>534.0686604268026</v>
       </c>
       <c r="D21" t="n">
-        <v>901.7423957773889</v>
+        <v>-204.3233814722879</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Wu</t>
+          <t>W</t>
         </is>
       </c>
       <c r="B22" t="n">
         <v>0</v>
       </c>
       <c r="C22" t="n">
-        <v>187.0092499959637</v>
+        <v>369.6548263151458</v>
       </c>
       <c r="D22" t="n">
-        <v>-816.5361814722879</v>
+        <v>700.6609782484265</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>Wu</t>
         </is>
       </c>
       <c r="B23" t="n">
         <v>0</v>
       </c>
       <c r="C23" t="n">
-        <v>347.059410430839</v>
+        <v>187.0092499959636</v>
       </c>
       <c r="D23" t="n">
-        <v>382.633</v>
+        <v>-586.9563814722879</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Mabs</t>
+          <t>U</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>0.6742997789701619</v>
+        <v>0</v>
       </c>
       <c r="C24" t="n">
-        <v>1.0361382500896</v>
+        <v>347.059410430839</v>
       </c>
       <c r="D24" t="n">
-        <v>1.49180779146426</v>
+        <v>382.633</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Mrel</t>
+          <t>Mabs</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>0</v>
+        <v>0.5023026870006502</v>
       </c>
       <c r="C25" t="n">
-        <v>0.6157633609201633</v>
+        <v>1.0361382500896</v>
       </c>
       <c r="D25" t="n">
-        <v>2.325308024035425</v>
+        <v>1.03853932146805</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>alpha</t>
+          <t>Mrel</t>
         </is>
       </c>
       <c r="B26" t="n">
         <v>0</v>
       </c>
       <c r="C26" t="n">
-        <v>59.16107092132572</v>
+        <v>0.6157633609201633</v>
       </c>
       <c r="D26" t="n">
-        <v>-48.59287643690928</v>
+        <v>1.677535710873892</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>beta</t>
+          <t>alpha</t>
         </is>
       </c>
       <c r="B27" t="n">
         <v>0</v>
       </c>
       <c r="C27" t="n">
-        <v>30.3912715428547</v>
+        <v>59.16107092132572</v>
       </c>
       <c r="D27" t="n">
-        <v>-64.89197315792033</v>
+        <v>-28.10190933351899</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>beta</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>1012.274989914663</v>
+        <v>0</v>
       </c>
       <c r="C28" t="n">
-        <v>766.1729229913674</v>
+        <v>30.39127154285467</v>
       </c>
       <c r="D28" t="n">
-        <v>491.9244548549424</v>
+        <v>-56.89993501062956</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>1012.274989914663</v>
+      </c>
+      <c r="C29" t="n">
+        <v>766.1729229913676</v>
+      </c>
+      <c r="D29" t="n">
+        <v>703.8595183369364</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
           <t>P</t>
         </is>
       </c>
-      <c r="B29" t="n">
-        <v>269971.8007849224</v>
-      </c>
-      <c r="C29" t="n">
-        <v>84445.80654685765</v>
-      </c>
-      <c r="D29" t="n">
-        <v>15707.09057984341</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr"/>
-      <c r="B30" t="inlineStr"/>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
+      <c r="B30" t="n">
+        <v>269.9718031524023</v>
+      </c>
+      <c r="C30" t="n">
+        <v>87.14554660265199</v>
+      </c>
+      <c r="D30" t="n">
+        <v>63.19544154522488</v>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr"/>
-      <c r="B31" t="inlineStr"/>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>reaction</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>0.615970303127865</v>
+      </c>
+      <c r="C31" t="n">
+        <v>0.615970303127865</v>
+      </c>
+      <c r="D31" t="n">
+        <v>0.615970303127865</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr"/>
@@ -883,236 +903,264 @@
       <c r="D32" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="1" t="inlineStr">
+      <c r="A33" t="inlineStr"/>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr"/>
+      <c r="B34" t="inlineStr"/>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="inlineStr">
         <is>
           <t>radius 2</t>
         </is>
       </c>
-      <c r="B33" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="C33" s="1" t="n">
+      <c r="B35" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D33" s="1" t="n">
+      <c r="D35" s="1" t="n">
         <v>2</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="B34" t="n">
-        <v>318.8608333333333</v>
-      </c>
-      <c r="C34" t="n">
-        <v>620.0166489913859</v>
-      </c>
-      <c r="D34" t="n">
-        <v>566.5365209390526</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Vax</t>
-        </is>
-      </c>
-      <c r="B35" t="n">
-        <v>318.8608333333333</v>
-      </c>
-      <c r="C35" t="n">
-        <v>318.8608333333333</v>
-      </c>
-      <c r="D35" t="n">
-        <v>382.633</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Vu</t>
+          <t>V</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>0</v>
+        <v>318.8608333333333</v>
       </c>
       <c r="C36" t="n">
-        <v>531.7409275130885</v>
+        <v>604.073894907561</v>
       </c>
       <c r="D36" t="n">
-        <v>-417.7985362213774</v>
+        <v>416.4996129834379</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>Vax</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>0</v>
+        <v>318.8608333333333</v>
       </c>
       <c r="C37" t="n">
-        <v>367.7235882130061</v>
+        <v>318.8608333333333</v>
       </c>
       <c r="D37" t="n">
-        <v>900.5151559555134</v>
+        <v>382.633</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Wu</t>
+          <t>Vu</t>
         </is>
       </c>
       <c r="B38" t="n">
         <v>0</v>
       </c>
       <c r="C38" t="n">
-        <v>183.1622403614367</v>
+        <v>513.0624128454191</v>
       </c>
       <c r="D38" t="n">
-        <v>-815.1806753208656</v>
+        <v>-164.5111392166304</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>W</t>
         </is>
       </c>
       <c r="B39" t="n">
         <v>0</v>
       </c>
       <c r="C39" t="n">
-        <v>348.5786871516519</v>
+        <v>353.1479371907907</v>
       </c>
       <c r="D39" t="n">
-        <v>397.3821390994881</v>
+        <v>745.4385302732458</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Mabs</t>
+          <t>Wu</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>0.6742997789701619</v>
+        <v>0</v>
       </c>
       <c r="C40" t="n">
-        <v>1.032810904743624</v>
+        <v>151.7933941516655</v>
       </c>
       <c r="D40" t="n">
-        <v>1.46091824474216</v>
+        <v>-639.7425964612148</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Mrel</t>
+          <t>U</t>
         </is>
       </c>
       <c r="B41" t="n">
         <v>0</v>
       </c>
       <c r="C41" t="n">
-        <v>0.6125463444500556</v>
+        <v>361.2690186937536</v>
       </c>
       <c r="D41" t="n">
-        <v>2.322143361246378</v>
+        <v>475.2314572445845</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>alpha</t>
+          <t>Mabs</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>0</v>
+        <v>0.5023026870006502</v>
       </c>
       <c r="C42" t="n">
-        <v>59.05080187210248</v>
+        <v>1.006253794872129</v>
       </c>
       <c r="D42" t="n">
-        <v>-47.51557056437037</v>
+        <v>0.997191218057449</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>beta</t>
+          <t>Mrel</t>
         </is>
       </c>
       <c r="B43" t="n">
         <v>0</v>
       </c>
       <c r="C43" t="n">
-        <v>29.87421848879016</v>
+        <v>0.5882665265710187</v>
       </c>
       <c r="D43" t="n">
-        <v>-64.85537720482064</v>
+        <v>1.784742969304252</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>alpha</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>1012.274989914663</v>
+        <v>0</v>
       </c>
       <c r="C44" t="n">
-        <v>768.3135147228602</v>
+        <v>58.13964945309809</v>
       </c>
       <c r="D44" t="n">
-        <v>504.4202355517214</v>
+        <v>-23.26504448048133</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" t="n">
+        <v>25.45673899364189</v>
+      </c>
+      <c r="D45" t="n">
+        <v>-59.11616134877179</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>1012.274989914663</v>
+      </c>
+      <c r="C46" t="n">
+        <v>785.1518038896713</v>
+      </c>
+      <c r="D46" t="n">
+        <v>717.0297207713031</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
           <t>P</t>
         </is>
       </c>
-      <c r="B45" t="n">
-        <v>269971.8007849224</v>
-      </c>
-      <c r="C45" t="n">
-        <v>85402.44743820207</v>
-      </c>
-      <c r="D45" t="n">
-        <v>17288.396942555</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr"/>
-      <c r="B46" t="inlineStr"/>
-      <c r="C46" t="inlineStr"/>
-      <c r="D46" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr"/>
-      <c r="B47" t="inlineStr"/>
-      <c r="C47" t="inlineStr"/>
-      <c r="D47" t="inlineStr"/>
+      <c r="B47" t="n">
+        <v>269.9718031524023</v>
+      </c>
+      <c r="C47" t="n">
+        <v>96.19486963079343</v>
+      </c>
+      <c r="D47" t="n">
+        <v>67.91377342006362</v>
+      </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr"/>
-      <c r="B48" t="inlineStr"/>
-      <c r="C48" t="inlineStr"/>
-      <c r="D48" t="inlineStr"/>
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>reaction</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>0.6300993702135176</v>
+      </c>
+      <c r="C48" t="n">
+        <v>0.6300993702135176</v>
+      </c>
+      <c r="D48" t="n">
+        <v>0.6300993702135176</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr"/>
       <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr"/>
+      <c r="B50" t="inlineStr"/>
+      <c r="C50" t="inlineStr"/>
+      <c r="D50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr"/>
+      <c r="B51" t="inlineStr"/>
+      <c r="C51" t="inlineStr"/>
+      <c r="D51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr"/>
+      <c r="B52" t="inlineStr"/>
+      <c r="C52" t="inlineStr"/>
+      <c r="D52" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1146,13 +1194,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.5393096058230218</v>
+        <v>0.53931</v>
       </c>
       <c r="C2" t="n">
-        <v>0.5393096058230218</v>
+        <v>0.53931</v>
       </c>
       <c r="D2" t="n">
-        <v>0.5393096058230218</v>
+        <v>0.53931</v>
       </c>
     </row>
     <row r="3">
@@ -1168,7 +1216,7 @@
         <v>1100</v>
       </c>
       <c r="D3" t="n">
-        <v>796.8223651450762</v>
+        <v>872.6167738588072</v>
       </c>
     </row>
     <row r="4">
@@ -1184,7 +1232,7 @@
         <v>789.0531605057781</v>
       </c>
       <c r="D4" t="n">
-        <v>491.9244548549424</v>
+        <v>703.8595183369364</v>
       </c>
     </row>
     <row r="5">
@@ -1194,13 +1242,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>377617.0666885399</v>
+        <v>377.61707</v>
       </c>
       <c r="C5" t="n">
-        <v>363701.0116931864</v>
+        <v>375.3285658578344</v>
       </c>
       <c r="D5" t="n">
-        <v>99330.44626184442</v>
+        <v>145.621235548294</v>
       </c>
     </row>
     <row r="6">
@@ -1210,13 +1258,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>269971.8007849224</v>
+        <v>269.9718031524023</v>
       </c>
       <c r="C6" t="n">
-        <v>95099.06001879823</v>
+        <v>98.13938554945281</v>
       </c>
       <c r="D6" t="n">
-        <v>15707.09057984341</v>
+        <v>63.19544154522488</v>
       </c>
     </row>
   </sheetData>
@@ -1230,7 +1278,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1251,13 +1299,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.2059260123647083</v>
+        <v>0.06628346485995232</v>
       </c>
       <c r="C2" t="n">
-        <v>0.2162223129829438</v>
+        <v>0.06959763810294993</v>
       </c>
       <c r="D2" t="n">
-        <v>0.2270334286320909</v>
+        <v>0.07307752000809743</v>
       </c>
     </row>
     <row r="3">
@@ -1267,13 +1315,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.2096262791747584</v>
+        <v>0.06820479360743238</v>
       </c>
       <c r="C3" t="n">
-        <v>0.2068274678141</v>
+        <v>0.06899730013328308</v>
       </c>
       <c r="D3" t="n">
-        <v>0.2357847585464695</v>
+        <v>0.0907625226398884</v>
       </c>
     </row>
     <row r="4">
@@ -1283,13 +1331,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.2022257455546583</v>
+        <v>0.06436213611247225</v>
       </c>
       <c r="C4" t="n">
-        <v>0.2050245569153167</v>
+        <v>0.06356962958662156</v>
       </c>
       <c r="D4" t="n">
-        <v>0.2182820987177123</v>
+        <v>0.05539251737630646</v>
       </c>
     </row>
     <row r="5">
@@ -1299,13 +1347,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.009575338020624545</v>
+        <v>0.001600356533626209</v>
       </c>
       <c r="C5" t="n">
-        <v>0.00233273465983992</v>
+        <v>0.002260468967924607</v>
       </c>
       <c r="D5" t="n">
-        <v>0.02496742353022317</v>
+        <v>0.01624047746882418</v>
       </c>
     </row>
     <row r="6">
@@ -1315,29 +1363,125 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>159</v>
+        <v>152</v>
       </c>
       <c r="C6" t="n">
-        <v>159</v>
+        <v>152</v>
       </c>
       <c r="D6" t="n">
-        <v>159</v>
+        <v>152</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
+          <t>stator cax</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0.0007861104377259694</v>
+      </c>
+      <c r="C7" t="n">
+        <v>-0.0008081196532425571</v>
+      </c>
+      <c r="D7" t="n">
+        <v>-0.002162873479156625</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>stator cm</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0.003090109347207215</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.003090109347207215</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.003090109347207215</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>stator stagger</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>30.10235297219402</v>
+      </c>
+      <c r="C9" t="n">
+        <v>29.58053546066286</v>
+      </c>
+      <c r="D9" t="n">
+        <v>29.06982472654904</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
           <t>rotor NOB</t>
         </is>
       </c>
-      <c r="B7" t="n">
-        <v>79</v>
-      </c>
-      <c r="C7" t="n">
-        <v>79</v>
-      </c>
-      <c r="D7" t="n">
-        <v>79</v>
+      <c r="B10" t="n">
+        <v>69</v>
+      </c>
+      <c r="C10" t="n">
+        <v>69</v>
+      </c>
+      <c r="D10" t="n">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>rotor cax</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>-0.005941224142767051</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.006942274807030737</v>
+      </c>
+      <c r="D11" t="n">
+        <v>-0.003901017033459622</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>rotor cm</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0.008986272204899438</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0.008986272204899438</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.008986272204899438</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>rotor stagger</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>-10.27323112066841</v>
+      </c>
+      <c r="C13" t="n">
+        <v>-13.25433173388744</v>
+      </c>
+      <c r="D13" t="n">
+        <v>-16.82971117756495</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added rotor disk design code.
also fixed station 2 calculations. static temperature was being
calculated with station 1 values.
</commit_message>
<xml_diff>
--- a/xjep_turbojet/turbine.xlsx
+++ b/xjep_turbojet/turbine.xlsx
@@ -456,10 +456,10 @@
         <v>318.8608333333333</v>
       </c>
       <c r="C2" t="n">
-        <v>641.6967391141203</v>
+        <v>617.0290198688851</v>
       </c>
       <c r="D2" t="n">
-        <v>468.048116610378</v>
+        <v>438.7651193133304</v>
       </c>
     </row>
     <row r="3">
@@ -488,10 +488,10 @@
         <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>556.8684530081297</v>
+        <v>528.2542762025967</v>
       </c>
       <c r="D4" t="n">
-        <v>-269.5570937176798</v>
+        <v>-214.7249804681354</v>
       </c>
     </row>
     <row r="5">
@@ -504,10 +504,10 @@
         <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>389.6878070433993</v>
+        <v>364.8754176398984</v>
       </c>
       <c r="D5" t="n">
-        <v>677.9017718664238</v>
+        <v>693.8614353100434</v>
       </c>
     </row>
     <row r="6">
@@ -520,10 +520,10 @@
         <v>0</v>
       </c>
       <c r="C6" t="n">
-        <v>224.0186508402053</v>
+        <v>177.3748555006106</v>
       </c>
       <c r="D6" t="n">
-        <v>-559.5916364730954</v>
+        <v>-578.8226660398791</v>
       </c>
     </row>
     <row r="7">
@@ -536,10 +536,10 @@
         <v>0</v>
       </c>
       <c r="C7" t="n">
-        <v>332.8498021679244</v>
+        <v>350.8794207019861</v>
       </c>
       <c r="D7" t="n">
-        <v>290.0345427554155</v>
+        <v>364.0976855717437</v>
       </c>
     </row>
     <row r="8">
@@ -552,10 +552,10 @@
         <v>0.5023026870006502</v>
       </c>
       <c r="C8" t="n">
-        <v>1.068925150273982</v>
+        <v>1.027834173970236</v>
       </c>
       <c r="D8" t="n">
-        <v>1.120609616342567</v>
+        <v>0.7948513250433605</v>
       </c>
     </row>
     <row r="9">
@@ -568,10 +568,10 @@
         <v>0</v>
       </c>
       <c r="C9" t="n">
-        <v>0.6491338857025494</v>
+        <v>0.6078019208426236</v>
       </c>
       <c r="D9" t="n">
-        <v>1.623045190290881</v>
+        <v>1.256974761612323</v>
       </c>
     </row>
     <row r="10">
@@ -584,10 +584,10 @@
         <v>0</v>
       </c>
       <c r="C10" t="n">
-        <v>60.20470594438805</v>
+        <v>58.88429813101271</v>
       </c>
       <c r="D10" t="n">
-        <v>-35.16390951060599</v>
+        <v>-29.30015432826924</v>
       </c>
     </row>
     <row r="11">
@@ -600,10 +600,10 @@
         <v>0</v>
       </c>
       <c r="C11" t="n">
-        <v>35.09031690804215</v>
+        <v>29.08616849183637</v>
       </c>
       <c r="D11" t="n">
-        <v>-55.63677914937897</v>
+        <v>-56.5331460007943</v>
       </c>
     </row>
     <row r="12">
@@ -616,10 +616,10 @@
         <v>1012.274989914663</v>
       </c>
       <c r="C12" t="n">
-        <v>744.7118374335867</v>
+        <v>771.5023603136317</v>
       </c>
       <c r="D12" t="n">
-        <v>676.1336498097077</v>
+        <v>699.9501327740873</v>
       </c>
     </row>
     <row r="13">
@@ -632,10 +632,10 @@
         <v>269.9718031524023</v>
       </c>
       <c r="C13" t="n">
-        <v>77.70112712892625</v>
+        <v>89.61901688602993</v>
       </c>
       <c r="D13" t="n">
-        <v>54.06219056033665</v>
+        <v>61.84297623748751</v>
       </c>
     </row>
     <row r="14">
@@ -645,13 +645,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.6276409011903206</v>
+        <v>0.63632777021812</v>
       </c>
       <c r="C14" t="n">
-        <v>0.6276409011903206</v>
+        <v>0.63632777021812</v>
       </c>
       <c r="D14" t="n">
-        <v>0.6276409011903206</v>
+        <v>0.63632777021812</v>
       </c>
     </row>
     <row r="15">
@@ -698,7 +698,7 @@
         <v>318.8608333333333</v>
       </c>
       <c r="C19" t="n">
-        <v>622.0141196822682</v>
+        <v>600.3196191516718</v>
       </c>
       <c r="D19" t="n">
         <v>433.7695896501622</v>
@@ -730,7 +730,7 @@
         <v>0</v>
       </c>
       <c r="C21" t="n">
-        <v>534.0686604268026</v>
+        <v>508.6368194540977</v>
       </c>
       <c r="D21" t="n">
         <v>-204.3233814722879</v>
@@ -746,7 +746,7 @@
         <v>0</v>
       </c>
       <c r="C22" t="n">
-        <v>369.6548263151458</v>
+        <v>349.9613117119709</v>
       </c>
       <c r="D22" t="n">
         <v>700.6609782484265</v>
@@ -762,7 +762,7 @@
         <v>0</v>
       </c>
       <c r="C23" t="n">
-        <v>187.0092499959636</v>
+        <v>144.2244385017167</v>
       </c>
       <c r="D23" t="n">
         <v>-586.9563814722879</v>
@@ -778,7 +778,7 @@
         <v>0</v>
       </c>
       <c r="C24" t="n">
-        <v>347.059410430839</v>
+        <v>364.4123809523809</v>
       </c>
       <c r="D24" t="n">
         <v>382.633</v>
@@ -794,10 +794,10 @@
         <v>0.5023026870006502</v>
       </c>
       <c r="C25" t="n">
-        <v>1.0361382500896</v>
+        <v>1</v>
       </c>
       <c r="D25" t="n">
-        <v>1.03853932146805</v>
+        <v>0.7858016007209785</v>
       </c>
     </row>
     <row r="26">
@@ -810,10 +810,10 @@
         <v>0</v>
       </c>
       <c r="C26" t="n">
-        <v>0.6157633609201633</v>
+        <v>0.5829583117848304</v>
       </c>
       <c r="D26" t="n">
-        <v>1.677535710873892</v>
+        <v>1.269292572387075</v>
       </c>
     </row>
     <row r="27">
@@ -826,7 +826,7 @@
         <v>0</v>
       </c>
       <c r="C27" t="n">
-        <v>59.16107092132572</v>
+        <v>57.91669106792425</v>
       </c>
       <c r="D27" t="n">
         <v>-28.10190933351899</v>
@@ -842,7 +842,7 @@
         <v>0</v>
       </c>
       <c r="C28" t="n">
-        <v>30.39127154285467</v>
+        <v>24.33778902887292</v>
       </c>
       <c r="D28" t="n">
         <v>-56.89993501062956</v>
@@ -858,7 +858,7 @@
         <v>1012.274989914663</v>
       </c>
       <c r="C29" t="n">
-        <v>766.1729229913676</v>
+        <v>789.0531605057781</v>
       </c>
       <c r="D29" t="n">
         <v>703.8595183369364</v>
@@ -874,7 +874,7 @@
         <v>269.9718031524023</v>
       </c>
       <c r="C30" t="n">
-        <v>87.14554660265199</v>
+        <v>98.13938554945281</v>
       </c>
       <c r="D30" t="n">
         <v>63.19544154522488</v>
@@ -887,13 +887,13 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>0.615970303127865</v>
+        <v>0.6672100461124595</v>
       </c>
       <c r="C31" t="n">
-        <v>0.615970303127865</v>
+        <v>0.6672100461124595</v>
       </c>
       <c r="D31" t="n">
-        <v>0.615970303127865</v>
+        <v>0.6672100461124595</v>
       </c>
     </row>
     <row r="32">
@@ -940,10 +940,10 @@
         <v>318.8608333333333</v>
       </c>
       <c r="C36" t="n">
-        <v>604.073894907561</v>
+        <v>584.9685121741846</v>
       </c>
       <c r="D36" t="n">
-        <v>416.4996129834379</v>
+        <v>429.4035172661643</v>
       </c>
     </row>
     <row r="37">
@@ -972,10 +972,10 @@
         <v>0</v>
       </c>
       <c r="C38" t="n">
-        <v>513.0624128454191</v>
+        <v>490.4242339049442</v>
       </c>
       <c r="D38" t="n">
-        <v>-164.5111392166304</v>
+        <v>-194.8829596233418</v>
       </c>
     </row>
     <row r="39">
@@ -988,10 +988,10 @@
         <v>0</v>
       </c>
       <c r="C39" t="n">
-        <v>353.1479371907907</v>
+        <v>338.1179266728307</v>
       </c>
       <c r="D39" t="n">
-        <v>745.4385302732458</v>
+        <v>708.2973485673466</v>
       </c>
     </row>
     <row r="40">
@@ -1004,10 +1004,10 @@
         <v>0</v>
       </c>
       <c r="C40" t="n">
-        <v>151.7933941516655</v>
+        <v>112.4788927021684</v>
       </c>
       <c r="D40" t="n">
-        <v>-639.7425964612148</v>
+        <v>-596.0512740515981</v>
       </c>
     </row>
     <row r="41">
@@ -1020,10 +1020,10 @@
         <v>0</v>
       </c>
       <c r="C41" t="n">
-        <v>361.2690186937536</v>
+        <v>377.9453412027758</v>
       </c>
       <c r="D41" t="n">
-        <v>475.2314572445845</v>
+        <v>401.1683144282563</v>
       </c>
     </row>
     <row r="42">
@@ -1036,10 +1036,10 @@
         <v>0.5023026870006502</v>
       </c>
       <c r="C42" t="n">
-        <v>1.006253794872129</v>
+        <v>0.974428443636108</v>
       </c>
       <c r="D42" t="n">
-        <v>0.997191218057449</v>
+        <v>0.7778921788756706</v>
       </c>
     </row>
     <row r="43">
@@ -1052,10 +1052,10 @@
         <v>0</v>
       </c>
       <c r="C43" t="n">
-        <v>0.5882665265710187</v>
+        <v>0.5632298460454024</v>
       </c>
       <c r="D43" t="n">
-        <v>1.784742969304252</v>
+        <v>1.283126349958124</v>
       </c>
     </row>
     <row r="44">
@@ -1068,10 +1068,10 @@
         <v>0</v>
       </c>
       <c r="C44" t="n">
-        <v>58.13964945309809</v>
+        <v>56.9691453258664</v>
       </c>
       <c r="D44" t="n">
-        <v>-23.26504448048133</v>
+        <v>-26.99069205934358</v>
       </c>
     </row>
     <row r="45">
@@ -1084,10 +1084,10 @@
         <v>0</v>
       </c>
       <c r="C45" t="n">
-        <v>25.45673899364189</v>
+        <v>19.43041121652287</v>
       </c>
       <c r="D45" t="n">
-        <v>-59.11616134877179</v>
+        <v>-57.3017097621832</v>
       </c>
     </row>
     <row r="46">
@@ -1100,10 +1100,10 @@
         <v>1012.274989914663</v>
       </c>
       <c r="C46" t="n">
-        <v>785.1518038896713</v>
+        <v>804.7526202343679</v>
       </c>
       <c r="D46" t="n">
-        <v>717.0297207713031</v>
+        <v>707.2396458430325</v>
       </c>
     </row>
     <row r="47">
@@ -1116,10 +1116,10 @@
         <v>269.9718031524023</v>
       </c>
       <c r="C47" t="n">
-        <v>96.19486963079343</v>
+        <v>106.264801564553</v>
       </c>
       <c r="D47" t="n">
-        <v>67.91377342006362</v>
+        <v>64.38240490405983</v>
       </c>
     </row>
     <row r="48">
@@ -1129,13 +1129,13 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>0.6300993702135176</v>
+        <v>0.6950865148639259</v>
       </c>
       <c r="C48" t="n">
-        <v>0.6300993702135176</v>
+        <v>0.6950865148639259</v>
       </c>
       <c r="D48" t="n">
-        <v>0.6300993702135176</v>
+        <v>0.6950865148639259</v>
       </c>
     </row>
     <row r="49">
@@ -1278,7 +1278,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1318,10 +1318,10 @@
         <v>0.06820479360743238</v>
       </c>
       <c r="C3" t="n">
-        <v>0.06899730013328308</v>
+        <v>0.0721822431251697</v>
       </c>
       <c r="D3" t="n">
-        <v>0.0907625226398884</v>
+        <v>0.07661750430372086</v>
       </c>
     </row>
     <row r="4">
@@ -1334,10 +1334,10 @@
         <v>0.06436213611247225</v>
       </c>
       <c r="C4" t="n">
-        <v>0.06356962958662156</v>
+        <v>0.06701303308073016</v>
       </c>
       <c r="D4" t="n">
-        <v>0.05539251737630646</v>
+        <v>0.06953753571247401</v>
       </c>
     </row>
     <row r="5">
@@ -1353,7 +1353,7 @@
         <v>0.002260468967924607</v>
       </c>
       <c r="D5" t="n">
-        <v>0.01624047746882418</v>
+        <v>0.003250835546369466</v>
       </c>
     </row>
     <row r="6">
@@ -1363,13 +1363,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>152</v>
+        <v>127</v>
       </c>
       <c r="C6" t="n">
-        <v>152</v>
+        <v>127</v>
       </c>
       <c r="D6" t="n">
-        <v>152</v>
+        <v>127</v>
       </c>
     </row>
     <row r="7">
@@ -1379,13 +1379,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.0007861104377259694</v>
+        <v>0.00321639626994978</v>
       </c>
       <c r="C7" t="n">
-        <v>-0.0008081196532425571</v>
+        <v>0.00323161114348426</v>
       </c>
       <c r="D7" t="n">
-        <v>-0.002162873479156625</v>
+        <v>0.003246287277403755</v>
       </c>
     </row>
     <row r="8">
@@ -1395,13 +1395,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.003090109347207215</v>
+        <v>0.003693388335819537</v>
       </c>
       <c r="C8" t="n">
-        <v>0.003090109347207215</v>
+        <v>0.003693388335819537</v>
       </c>
       <c r="D8" t="n">
-        <v>0.003090109347207215</v>
+        <v>0.003693388335819537</v>
       </c>
     </row>
     <row r="9">
@@ -1411,13 +1411,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>30.10235297219402</v>
+        <v>29.44214906550635</v>
       </c>
       <c r="C9" t="n">
-        <v>29.58053546066286</v>
+        <v>28.95834553396212</v>
       </c>
       <c r="D9" t="n">
-        <v>29.06982472654904</v>
+        <v>28.4845726629332</v>
       </c>
     </row>
     <row r="10">
@@ -1427,13 +1427,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>69</v>
+        <v>101</v>
       </c>
       <c r="C10" t="n">
-        <v>69</v>
+        <v>101</v>
       </c>
       <c r="D10" t="n">
-        <v>69</v>
+        <v>101</v>
       </c>
     </row>
     <row r="11">
@@ -1443,13 +1443,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>-0.005941224142767051</v>
+        <v>0.005949744205854119</v>
       </c>
       <c r="C11" t="n">
-        <v>0.006942274807030737</v>
+        <v>0.005878980759330096</v>
       </c>
       <c r="D11" t="n">
-        <v>-0.003901017033459622</v>
+        <v>0.005793148808102232</v>
       </c>
     </row>
     <row r="12">
@@ -1459,13 +1459,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.008986272204899438</v>
+        <v>0.00612458931784321</v>
       </c>
       <c r="C12" t="n">
-        <v>0.008986272204899438</v>
+        <v>0.00612458931784321</v>
       </c>
       <c r="D12" t="n">
-        <v>0.008986272204899438</v>
+        <v>0.00612458931784321</v>
       </c>
     </row>
     <row r="13">
@@ -1475,13 +1475,29 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>-10.27323112066841</v>
+        <v>-13.72348875447896</v>
       </c>
       <c r="C13" t="n">
-        <v>-13.25433173388744</v>
+        <v>-16.28107299087832</v>
       </c>
       <c r="D13" t="n">
-        <v>-16.82971117756495</v>
+        <v>-18.93564927283017</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>axial spacing</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0.00482459440492467</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.00482459440492467</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.00482459440492467</v>
       </c>
     </row>
   </sheetData>

</xml_diff>